<commit_message>
test(e2e): loading skeleton 表示を20画面で実機検証（GET 1.2s 遅延注入・20/20 PASS）
spec 正本の「データ取得 loading」20行を PASS 化し xlsx 再生成。
</commit_message>
<xml_diff>
--- a/apps/web/.qa/テスト仕様書_エンジニア版.xlsx
+++ b/apps/web/.qa/テスト仕様書_エンジニア版.xlsx
@@ -1,39 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="概要" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SA01_サインインサインアップ" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SA03_ワークスペース設定" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SB01_プロジェクト一覧" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SB02_プロジェクトダッシュボード" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SC01_AI社員 組織図" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SC02_AI社員 編集" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SF01_工程ワークフロー(司令塔)" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SF02_フェーズ管理" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SG01_成果物ビューア" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SH01_モックビューア" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SI01_タスクボード" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SI02_タスク詳細(6タブ)" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SI03_実行モニタ(SSE)" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SJ01_承認インボックス" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SK01_ナレッジエクスプローラ" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SK02_昇格レビュー" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SL01_クライアント招待管理" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SL02_クライアントサインイン" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SL03_クライアントプロジェクトビュー" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SM01_議事録アップロード" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SO01_自動スケジュール(cron)" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TUC36_通知センター" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TUC37_プロフィール" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TUC38_ワークスペース切替" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TUC39_プロジェクト切替" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TUC40_グローバル検索" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="概要" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="SA01_サインインサインアップ" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="SA03_ワークスペース設定" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="SB01_プロジェクト一覧" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="SB02_プロジェクトダッシュボード" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="SC01_AI社員 組織図" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="SC02_AI社員 編集" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="SF01_工程ワークフロー(司令塔)" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="SF02_フェーズ管理" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="SG01_成果物ビューア" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="SH01_モックビューア" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="SI01_タスクボード" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="SI02_タスク詳細(6タブ)" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="SI03_実行モニタ(SSE)" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="SJ01_承認インボックス" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="SK01_ナレッジエクスプローラ" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="SK02_昇格レビュー" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="SL01_クライアント招待管理" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="SL02_クライアントサインイン" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="SL03_クライアントプロジェクトビュー" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="SM01_議事録アップロード" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="SO01_自動スケジュール(cron)" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="TUC36_通知センター" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="TUC37_プロフィール" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="TUC38_ワークスペース切替" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="TUC39_プロジェクト切替" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="TUC40_グローバル検索" sheetId="27" state="visible" r:id="rId27"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -583,13 +583,13 @@
         <v>18</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D6" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7">
@@ -621,13 +621,13 @@
         <v>12</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D8" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9">
@@ -640,13 +640,13 @@
         <v>12</v>
       </c>
       <c r="C9" s="3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D9" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10">
@@ -659,13 +659,13 @@
         <v>17</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D10" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11">
@@ -678,13 +678,13 @@
         <v>11</v>
       </c>
       <c r="C11" s="3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D11" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
@@ -697,13 +697,13 @@
         <v>14</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D12" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13">
@@ -716,13 +716,13 @@
         <v>25</v>
       </c>
       <c r="C13" s="3" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D13" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14">
@@ -735,13 +735,13 @@
         <v>17</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D14" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15">
@@ -754,13 +754,13 @@
         <v>14</v>
       </c>
       <c r="C15" s="3" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D15" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="16">
@@ -773,13 +773,13 @@
         <v>24</v>
       </c>
       <c r="C16" s="3" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D16" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
     <row r="17">
@@ -830,13 +830,13 @@
         <v>11</v>
       </c>
       <c r="C19" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D19" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="20">
@@ -849,13 +849,13 @@
         <v>16</v>
       </c>
       <c r="C20" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D20" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="21">
@@ -868,13 +868,13 @@
         <v>18</v>
       </c>
       <c r="C21" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D21" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="22">
@@ -944,13 +944,13 @@
         <v>15</v>
       </c>
       <c r="C25" s="3" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D25" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E25" s="3" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="26">
@@ -982,13 +982,13 @@
         <v>19</v>
       </c>
       <c r="C27" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D27" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="28">
@@ -1001,13 +1001,13 @@
         <v>11</v>
       </c>
       <c r="C28" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D28" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="29">
@@ -1020,13 +1020,13 @@
         <v>11</v>
       </c>
       <c r="C29" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D29" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="30">
@@ -1207,43 +1207,47 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>SG01-003</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>成果物ビューア</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>データ取得</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>loading skeleton 表示（成果物メタ）</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>取得未完</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>1. 成果物ビューア を開き取得完了前を観察</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>&lt;Loading&gt;（role=status/aria-live）が出る</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr"/>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -1383,43 +1387,47 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>SG01-007</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>成果物ビューア</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>データ取得</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>loading skeleton 表示（署名DL URL）</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>取得未完</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>1. 成果物ビューア を開き取得完了前を観察</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr">
         <is>
           <t>&lt;Loading&gt;（role=status/aria-live）が出る</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr"/>
-      <c r="I8" s="3" t="inlineStr"/>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -1559,43 +1567,47 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>SG01-011</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>成果物ビューア</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>データ取得</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>loading skeleton 表示（コメント）</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>取得未完</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="F12" s="4" t="inlineStr">
         <is>
           <t>1. 成果物ビューア を開き取得完了前を観察</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr">
+      <c r="G12" s="4" t="inlineStr">
         <is>
           <t>&lt;Loading&gt;（role=status/aria-live）が出る</t>
         </is>
       </c>
-      <c r="H12" s="3" t="inlineStr"/>
-      <c r="I12" s="3" t="inlineStr"/>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -2382,43 +2394,47 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>SH01-003</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>モックビューア</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>データ取得</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>loading skeleton 表示（モック詳細）</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>取得未完</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>1. モックビューア を開き取得完了前を観察</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>&lt;Loading&gt;（role=status/aria-live）が出る</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr"/>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -2554,43 +2570,47 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>SH01-007</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>モックビューア</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>データ取得</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>loading skeleton 表示（署名DL URL）</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>取得未完</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>1. モックビューア を開き取得完了前を観察</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr">
         <is>
           <t>&lt;Loading&gt;（role=status/aria-live）が出る</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr"/>
-      <c r="I8" s="3" t="inlineStr"/>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -3197,43 +3217,47 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>SI01-003</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>タスクボード</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>データ取得</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>loading skeleton 表示（タスク一覧）</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>取得未完</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>1. タスクボード を開き取得完了前を観察</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>&lt;Loading&gt;（role=status/aria-live）が出る</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr"/>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -3895,43 +3919,47 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>SI02-003</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>タスク詳細(6タブ)</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>データ取得</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>loading skeleton 表示（詳細）</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>取得未完</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>1. タスク詳細(6タブ) を開き取得完了前を観察</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>&lt;Loading&gt;（role=status/aria-live）が出る</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr"/>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -4071,43 +4099,47 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>SI02-007</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>タスク詳細(6タブ)</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>データ取得</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>loading skeleton 表示（受入条件）</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>取得未完</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>1. タスク詳細(6タブ) を開き取得完了前を観察</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr">
         <is>
           <t>&lt;Loading&gt;（role=status/aria-live）が出る</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr"/>
-      <c r="I8" s="3" t="inlineStr"/>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -4247,43 +4279,47 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>SI02-011</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>タスク詳細(6タブ)</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>データ取得</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>loading skeleton 表示（実行履歴）</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>取得未完</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="F12" s="4" t="inlineStr">
         <is>
           <t>1. タスク詳細(6タブ) を開き取得完了前を観察</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr">
+      <c r="G12" s="4" t="inlineStr">
         <is>
           <t>&lt;Loading&gt;（role=status/aria-live）が出る</t>
         </is>
       </c>
-      <c r="H12" s="3" t="inlineStr"/>
-      <c r="I12" s="3" t="inlineStr"/>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -4423,43 +4459,47 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>SI02-015</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>タスク詳細(6タブ)</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>データ取得</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>loading skeleton 表示（コメント）</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="E16" s="4" t="inlineStr">
         <is>
           <t>取得未完</t>
         </is>
       </c>
-      <c r="F16" s="3" t="inlineStr">
+      <c r="F16" s="4" t="inlineStr">
         <is>
           <t>1. タスク詳細(6タブ) を開き取得完了前を観察</t>
         </is>
       </c>
-      <c r="G16" s="3" t="inlineStr">
+      <c r="G16" s="4" t="inlineStr">
         <is>
           <t>&lt;Loading&gt;（role=status/aria-live）が出る</t>
         </is>
       </c>
-      <c r="H16" s="3" t="inlineStr"/>
-      <c r="I16" s="3" t="inlineStr"/>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I16" s="4" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -6376,43 +6416,47 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>SK01-003</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>ナレッジエクスプローラ</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>データ取得</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>loading skeleton 表示（ナレッジツリー）</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>取得未完</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>1. ナレッジエクスプローラ を開き取得完了前を観察</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>&lt;Loading&gt;（role=status/aria-live）が出る</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr"/>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -6933,43 +6977,47 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>SK02-003</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>昇格レビュー</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>データ取得</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>loading skeleton 表示（昇格候補）</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>取得未完</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>1. 昇格レビュー を開き取得完了前を観察</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>&lt;Loading&gt;（role=status/aria-live）が出る</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr"/>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -7705,43 +7753,47 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>SL01-003</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>クライアント招待管理</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>データ取得</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>loading skeleton 表示（招待一覧）</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>取得未完</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>1. クライアント招待管理 を開き取得完了前を観察</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>&lt;Loading&gt;（role=status/aria-live）が出る</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr"/>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -11326,43 +11378,47 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>SO01-003</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>自動スケジュール(cron)</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>データ取得</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>loading skeleton 表示（スケジュール一覧）</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>取得未完</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>1. 自動スケジュール(cron) を開き取得完了前を観察</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>&lt;Loading&gt;（role=status/aria-live）が出る</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr"/>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -12855,43 +12911,47 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>TUC37-003</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>プロフィール</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>データ取得</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>loading skeleton 表示（自己プロフィール）</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>取得未完</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>1. プロフィール を開き取得完了前を観察</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>&lt;Loading&gt;（role=status/aria-live）が出る</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr"/>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -13736,43 +13796,47 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>TUC38-003</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>ワークスペース切替</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>データ取得</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>loading skeleton 表示（所属 WS 一覧）</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>取得未完</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>1. ワークスペース切替 を開き取得完了前を観察</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>&lt;Loading&gt;（role=status/aria-live）が出る</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr"/>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -14293,43 +14357,47 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>TUC39-003</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>プロジェクト切替</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>データ取得</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>loading skeleton 表示（現在WS内プロジェクト）</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>取得未完</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>1. プロジェクト切替 を開き取得完了前を観察</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>&lt;Loading&gt;（role=status/aria-live）が出る</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr"/>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -15583,43 +15651,47 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>SA03-003</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>ワークスペース設定</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>データ取得</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>loading skeleton 表示（WS 詳細）</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>取得未完</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>1. ワークスペース設定 を開き取得完了前を観察</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>&lt;Loading&gt;（role=status/aria-live）が出る</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr"/>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -17096,43 +17168,47 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>SB02-003</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>プロジェクトダッシュボード</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>データ取得</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>loading skeleton 表示（KPI ダッシュボード）</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>取得未完</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>1. プロジェクトダッシュボード を開き取得完了前を観察</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>&lt;Loading&gt;（role=status/aria-live）が出る</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr"/>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -17704,43 +17780,47 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>SC01-003</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>AI社員 組織図</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>データ取得</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>loading skeleton 表示（AI 社員一覧）</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>取得未完</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>1. AI社員 組織図 を開き取得完了前を観察</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>&lt;Loading&gt;（role=status/aria-live）が出る</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr"/>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -18312,43 +18392,47 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>SC02-003</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>AI社員 編集</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>データ取得</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>loading skeleton 表示（社員詳細）</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>取得未完</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>1. AI社員 編集 を開き取得完了前を観察</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>&lt;Loading&gt;（role=status/aria-live）が出る</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr"/>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -19119,43 +19203,47 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>SF01-003</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>工程ワークフロー(司令塔)</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>データ取得</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>loading skeleton 表示（工程一覧）</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>取得未完</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>1. 工程ワークフロー(司令塔) を開き取得完了前を観察</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>&lt;Loading&gt;（role=status/aria-live）が出る</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr"/>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -19680,43 +19768,47 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>SF02-003</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>フェーズ管理</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>データ取得</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>loading skeleton 表示（工程一覧）</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>取得未完</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>1. フェーズ管理 を開き取得完了前を観察</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>&lt;Loading&gt;（role=status/aria-live）が出る</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr"/>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">

</xml_diff>

<commit_message>
test(e2e): loading skeleton 表示を20画面で実機検証（GET 1.2s 遅延注入・20/20 PASS） (#257)
spec 正本の「データ取得 loading」20行を PASS 化し xlsx 再生成。

Co-authored-by: Atelier <info@engine-base.com>
</commit_message>
<xml_diff>
--- a/apps/web/.qa/テスト仕様書_エンジニア版.xlsx
+++ b/apps/web/.qa/テスト仕様書_エンジニア版.xlsx
@@ -1,39 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="概要" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SA01_サインインサインアップ" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SA03_ワークスペース設定" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SB01_プロジェクト一覧" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SB02_プロジェクトダッシュボード" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SC01_AI社員 組織図" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SC02_AI社員 編集" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SF01_工程ワークフロー(司令塔)" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SF02_フェーズ管理" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SG01_成果物ビューア" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SH01_モックビューア" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SI01_タスクボード" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SI02_タスク詳細(6タブ)" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SI03_実行モニタ(SSE)" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SJ01_承認インボックス" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SK01_ナレッジエクスプローラ" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SK02_昇格レビュー" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SL01_クライアント招待管理" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SL02_クライアントサインイン" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SL03_クライアントプロジェクトビュー" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SM01_議事録アップロード" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SO01_自動スケジュール(cron)" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TUC36_通知センター" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TUC37_プロフィール" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TUC38_ワークスペース切替" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TUC39_プロジェクト切替" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TUC40_グローバル検索" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="概要" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="SA01_サインインサインアップ" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="SA03_ワークスペース設定" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="SB01_プロジェクト一覧" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="SB02_プロジェクトダッシュボード" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="SC01_AI社員 組織図" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="SC02_AI社員 編集" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="SF01_工程ワークフロー(司令塔)" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="SF02_フェーズ管理" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="SG01_成果物ビューア" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="SH01_モックビューア" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="SI01_タスクボード" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="SI02_タスク詳細(6タブ)" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="SI03_実行モニタ(SSE)" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="SJ01_承認インボックス" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="SK01_ナレッジエクスプローラ" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="SK02_昇格レビュー" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="SL01_クライアント招待管理" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="SL02_クライアントサインイン" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="SL03_クライアントプロジェクトビュー" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="SM01_議事録アップロード" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="SO01_自動スケジュール(cron)" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="TUC36_通知センター" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="TUC37_プロフィール" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="TUC38_ワークスペース切替" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="TUC39_プロジェクト切替" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="TUC40_グローバル検索" sheetId="27" state="visible" r:id="rId27"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -583,13 +583,13 @@
         <v>18</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D6" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7">
@@ -621,13 +621,13 @@
         <v>12</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D8" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9">
@@ -640,13 +640,13 @@
         <v>12</v>
       </c>
       <c r="C9" s="3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D9" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10">
@@ -659,13 +659,13 @@
         <v>17</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D10" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11">
@@ -678,13 +678,13 @@
         <v>11</v>
       </c>
       <c r="C11" s="3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D11" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
@@ -697,13 +697,13 @@
         <v>14</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D12" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13">
@@ -716,13 +716,13 @@
         <v>25</v>
       </c>
       <c r="C13" s="3" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D13" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14">
@@ -735,13 +735,13 @@
         <v>17</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D14" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15">
@@ -754,13 +754,13 @@
         <v>14</v>
       </c>
       <c r="C15" s="3" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D15" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="16">
@@ -773,13 +773,13 @@
         <v>24</v>
       </c>
       <c r="C16" s="3" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D16" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
     <row r="17">
@@ -830,13 +830,13 @@
         <v>11</v>
       </c>
       <c r="C19" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D19" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="20">
@@ -849,13 +849,13 @@
         <v>16</v>
       </c>
       <c r="C20" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D20" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="21">
@@ -868,13 +868,13 @@
         <v>18</v>
       </c>
       <c r="C21" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D21" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="22">
@@ -944,13 +944,13 @@
         <v>15</v>
       </c>
       <c r="C25" s="3" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D25" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E25" s="3" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="26">
@@ -982,13 +982,13 @@
         <v>19</v>
       </c>
       <c r="C27" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D27" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="28">
@@ -1001,13 +1001,13 @@
         <v>11</v>
       </c>
       <c r="C28" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D28" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="29">
@@ -1020,13 +1020,13 @@
         <v>11</v>
       </c>
       <c r="C29" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D29" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="30">
@@ -1207,43 +1207,47 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>SG01-003</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>成果物ビューア</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>データ取得</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>loading skeleton 表示（成果物メタ）</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>取得未完</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>1. 成果物ビューア を開き取得完了前を観察</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>&lt;Loading&gt;（role=status/aria-live）が出る</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr"/>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -1383,43 +1387,47 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>SG01-007</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>成果物ビューア</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>データ取得</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>loading skeleton 表示（署名DL URL）</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>取得未完</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>1. 成果物ビューア を開き取得完了前を観察</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr">
         <is>
           <t>&lt;Loading&gt;（role=status/aria-live）が出る</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr"/>
-      <c r="I8" s="3" t="inlineStr"/>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -1559,43 +1567,47 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>SG01-011</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>成果物ビューア</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>データ取得</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>loading skeleton 表示（コメント）</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>取得未完</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="F12" s="4" t="inlineStr">
         <is>
           <t>1. 成果物ビューア を開き取得完了前を観察</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr">
+      <c r="G12" s="4" t="inlineStr">
         <is>
           <t>&lt;Loading&gt;（role=status/aria-live）が出る</t>
         </is>
       </c>
-      <c r="H12" s="3" t="inlineStr"/>
-      <c r="I12" s="3" t="inlineStr"/>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -2382,43 +2394,47 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>SH01-003</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>モックビューア</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>データ取得</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>loading skeleton 表示（モック詳細）</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>取得未完</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>1. モックビューア を開き取得完了前を観察</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>&lt;Loading&gt;（role=status/aria-live）が出る</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr"/>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -2554,43 +2570,47 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>SH01-007</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>モックビューア</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>データ取得</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>loading skeleton 表示（署名DL URL）</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>取得未完</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>1. モックビューア を開き取得完了前を観察</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr">
         <is>
           <t>&lt;Loading&gt;（role=status/aria-live）が出る</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr"/>
-      <c r="I8" s="3" t="inlineStr"/>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -3197,43 +3217,47 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>SI01-003</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>タスクボード</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>データ取得</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>loading skeleton 表示（タスク一覧）</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>取得未完</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>1. タスクボード を開き取得完了前を観察</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>&lt;Loading&gt;（role=status/aria-live）が出る</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr"/>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -3895,43 +3919,47 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>SI02-003</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>タスク詳細(6タブ)</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>データ取得</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>loading skeleton 表示（詳細）</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>取得未完</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>1. タスク詳細(6タブ) を開き取得完了前を観察</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>&lt;Loading&gt;（role=status/aria-live）が出る</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr"/>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -4071,43 +4099,47 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>SI02-007</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>タスク詳細(6タブ)</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>データ取得</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>loading skeleton 表示（受入条件）</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>取得未完</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>1. タスク詳細(6タブ) を開き取得完了前を観察</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr">
         <is>
           <t>&lt;Loading&gt;（role=status/aria-live）が出る</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr"/>
-      <c r="I8" s="3" t="inlineStr"/>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -4247,43 +4279,47 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>SI02-011</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>タスク詳細(6タブ)</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>データ取得</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>loading skeleton 表示（実行履歴）</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>取得未完</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="F12" s="4" t="inlineStr">
         <is>
           <t>1. タスク詳細(6タブ) を開き取得完了前を観察</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr">
+      <c r="G12" s="4" t="inlineStr">
         <is>
           <t>&lt;Loading&gt;（role=status/aria-live）が出る</t>
         </is>
       </c>
-      <c r="H12" s="3" t="inlineStr"/>
-      <c r="I12" s="3" t="inlineStr"/>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -4423,43 +4459,47 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>SI02-015</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>タスク詳細(6タブ)</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>データ取得</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>loading skeleton 表示（コメント）</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="E16" s="4" t="inlineStr">
         <is>
           <t>取得未完</t>
         </is>
       </c>
-      <c r="F16" s="3" t="inlineStr">
+      <c r="F16" s="4" t="inlineStr">
         <is>
           <t>1. タスク詳細(6タブ) を開き取得完了前を観察</t>
         </is>
       </c>
-      <c r="G16" s="3" t="inlineStr">
+      <c r="G16" s="4" t="inlineStr">
         <is>
           <t>&lt;Loading&gt;（role=status/aria-live）が出る</t>
         </is>
       </c>
-      <c r="H16" s="3" t="inlineStr"/>
-      <c r="I16" s="3" t="inlineStr"/>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I16" s="4" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -6376,43 +6416,47 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>SK01-003</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>ナレッジエクスプローラ</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>データ取得</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>loading skeleton 表示（ナレッジツリー）</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>取得未完</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>1. ナレッジエクスプローラ を開き取得完了前を観察</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>&lt;Loading&gt;（role=status/aria-live）が出る</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr"/>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -6933,43 +6977,47 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>SK02-003</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>昇格レビュー</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>データ取得</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>loading skeleton 表示（昇格候補）</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>取得未完</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>1. 昇格レビュー を開き取得完了前を観察</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>&lt;Loading&gt;（role=status/aria-live）が出る</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr"/>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -7705,43 +7753,47 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>SL01-003</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>クライアント招待管理</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>データ取得</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>loading skeleton 表示（招待一覧）</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>取得未完</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>1. クライアント招待管理 を開き取得完了前を観察</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>&lt;Loading&gt;（role=status/aria-live）が出る</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr"/>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -11326,43 +11378,47 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>SO01-003</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>自動スケジュール(cron)</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>データ取得</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>loading skeleton 表示（スケジュール一覧）</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>取得未完</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>1. 自動スケジュール(cron) を開き取得完了前を観察</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>&lt;Loading&gt;（role=status/aria-live）が出る</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr"/>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -12855,43 +12911,47 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>TUC37-003</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>プロフィール</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>データ取得</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>loading skeleton 表示（自己プロフィール）</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>取得未完</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>1. プロフィール を開き取得完了前を観察</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>&lt;Loading&gt;（role=status/aria-live）が出る</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr"/>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -13736,43 +13796,47 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>TUC38-003</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>ワークスペース切替</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>データ取得</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>loading skeleton 表示（所属 WS 一覧）</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>取得未完</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>1. ワークスペース切替 を開き取得完了前を観察</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>&lt;Loading&gt;（role=status/aria-live）が出る</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr"/>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -14293,43 +14357,47 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>TUC39-003</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>プロジェクト切替</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>データ取得</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>loading skeleton 表示（現在WS内プロジェクト）</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>取得未完</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>1. プロジェクト切替 を開き取得完了前を観察</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>&lt;Loading&gt;（role=status/aria-live）が出る</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr"/>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -15583,43 +15651,47 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>SA03-003</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>ワークスペース設定</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>データ取得</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>loading skeleton 表示（WS 詳細）</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>取得未完</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>1. ワークスペース設定 を開き取得完了前を観察</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>&lt;Loading&gt;（role=status/aria-live）が出る</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr"/>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -17096,43 +17168,47 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>SB02-003</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>プロジェクトダッシュボード</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>データ取得</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>loading skeleton 表示（KPI ダッシュボード）</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>取得未完</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>1. プロジェクトダッシュボード を開き取得完了前を観察</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>&lt;Loading&gt;（role=status/aria-live）が出る</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr"/>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -17704,43 +17780,47 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>SC01-003</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>AI社員 組織図</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>データ取得</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>loading skeleton 表示（AI 社員一覧）</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>取得未完</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>1. AI社員 組織図 を開き取得完了前を観察</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>&lt;Loading&gt;（role=status/aria-live）が出る</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr"/>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -18312,43 +18392,47 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>SC02-003</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>AI社員 編集</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>データ取得</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>loading skeleton 表示（社員詳細）</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>取得未完</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>1. AI社員 編集 を開き取得完了前を観察</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>&lt;Loading&gt;（role=status/aria-live）が出る</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr"/>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -19119,43 +19203,47 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>SF01-003</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>工程ワークフロー(司令塔)</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>データ取得</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>loading skeleton 表示（工程一覧）</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>取得未完</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>1. 工程ワークフロー(司令塔) を開き取得完了前を観察</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>&lt;Loading&gt;（role=status/aria-live）が出る</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr"/>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -19680,43 +19768,47 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>SF02-003</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>フェーズ管理</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>データ取得</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>loading skeleton 表示（工程一覧）</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>取得未完</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>1. フェーズ管理 を開き取得完了前を観察</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>&lt;Loading&gt;（role=status/aria-live）が出る</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr"/>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">

</xml_diff>

<commit_message>
test(e2e): フィールドバリデーション実機検証（signup zod 3種 + L02 token・4/4 PASS） (#258)
spec の S-A01/S-L02 バリデーション行を PASS 化し xlsx 再生成。

Co-authored-by: Atelier <info@engine-base.com>
</commit_message>
<xml_diff>
--- a/apps/web/.qa/テスト仕様書_エンジニア版.xlsx
+++ b/apps/web/.qa/テスト仕様書_エンジニア版.xlsx
@@ -564,13 +564,13 @@
         <v>16</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D5" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6">
@@ -887,13 +887,13 @@
         <v>14</v>
       </c>
       <c r="C22" s="3" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D22" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="23">
@@ -8658,43 +8658,47 @@
       <c r="I4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>SL02-004</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>クライアントサインイン</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>バリデーション</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>招待トークン: 必須/最小10</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>1. 招待トークン に不正値/未入力を入れる</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>エラー表示 かつ 送信ボタン無効</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr"/>
-      <c r="I5" s="3" t="inlineStr"/>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -8740,43 +8744,47 @@
       <c r="I6" s="4" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>SL02-006</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>クライアントサインイン</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>バリデーション</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>表示名: 任意</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>1. 表示名 に不正値/未入力を入れる</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G7" s="4" t="inlineStr">
         <is>
           <t>エラー表示 かつ 送信ボタン無効</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr"/>
-      <c r="I7" s="3" t="inlineStr"/>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -9336,43 +9344,47 @@
       <c r="I4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>SA01-004</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>サインイン/サインアップ</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>バリデーション</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>email: 必須/型/最大200</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>1. email に不正値/未入力を入れる</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>エラー表示 かつ 送信ボタン無効</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr"/>
-      <c r="I5" s="3" t="inlineStr"/>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -9414,43 +9426,47 @@
       <c r="I6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>SA01-006</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>サインイン/サインアップ</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>バリデーション</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>password: 必須/型</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>1. password に不正値/未入力を入れる</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G7" s="4" t="inlineStr">
         <is>
           <t>エラー表示 かつ 送信ボタン無効</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr"/>
-      <c r="I7" s="3" t="inlineStr"/>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">

</xml_diff>